<commit_message>
Replace bank with Mao overview dual scopes
</commit_message>
<xml_diff>
--- a/题库导入模板.xlsx
+++ b/题库导入模板.xlsx
@@ -423,304 +423,220 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="50" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="46" customWidth="1" min="12" max="12"/>
-    <col width="24" customWidth="1" min="13" max="13"/>
-    <col width="24" customWidth="1" min="14" max="14"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="56" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="56" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>难度层级</t>
+          <t>章节</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>知识分类</t>
+          <t>题型</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>题型</t>
+          <t>题干</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>题干</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>选项A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>选项B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>选项C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>选项D</t>
+          <t>正确答案</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>选项E</t>
+          <t>解析</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>选项F</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>标准答案</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>解析</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>知识点标签</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>来源/依据</t>
+          <t>易错点标签</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>基础层</t>
+          <t>导论 马克思主义中国化时代化</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>M1 大模型基础概念/Token</t>
+          <t>单选</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>单选</t>
+          <t>马克思主义中国化第一次历史性飞跃产生的理论成果是（ ）。</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Token 通常指什么？</t>
+          <t>毛泽东思想</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>最小语义/文本切分单元</t>
+          <t>邓小平理论</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>模型参数</t>
+          <t>“三个代表”重要思想</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>数据库表</t>
+          <t>科学发展观</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>网络协议</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
-        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>Token 是模型处理文本的基本切分单元。</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>Token、基础概念</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>毛泽东思想是马克思主义中国化第一次历史性飞跃的理论成果。</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>第一次飞跃</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>进阶层</t>
+          <t>第一章 毛泽东思想及其历史地位</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>M3 提示词工程/结构化提示</t>
+          <t>多选</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>多选</t>
+          <t>毛泽东思想活的灵魂包括（ ）。</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>以下属于结构化提示词常见要素的是？</t>
+          <t>实事求是</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>角色</t>
+          <t>群众路线</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>任务</t>
+          <t>独立自主</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>约束</t>
+          <t>依法治国</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>输出格式</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>ABCD</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>结构化提示一般包含角色、任务、约束和输出格式。</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>提示词工程</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr"/>
+          <t>ABC</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>实事求是、群众路线、独立自主是毛泽东思想活的灵魂。</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>活的灵魂</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>基础层</t>
+          <t>第二章 新民主主义革命理论</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>M1 大模型基础概念/判断</t>
+          <t>判断</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>判断</t>
+          <t>新民主主义革命是无产阶级领导的人民大众的反帝反封建革命。</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>大模型输出一定完全准确。</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr"/>
+          <t>正确</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>错误</t>
+        </is>
+      </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>错</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>大模型存在幻觉风险。</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>能力边界</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>冲刺层</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>场景案例专项/综合分析</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>简答</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>简述企业落地 RAG 时应关注的关键环节。</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>参考答案：知识库清洗、切分、向量化、召回、重排、权限与评测。</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>围绕数据治理、检索质量和安全合规展开。</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>RAG、落地实践</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>正确</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>新民主主义革命领导阶级是无产阶级。</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>革命性质</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -733,7 +649,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -761,7 +677,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>难度层级</t>
+          <t>章节</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -771,14 +687,14 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>只能填写：基础层、进阶层、冲刺层</t>
+          <t>章节名称，可用 / 分隔多级分类，例如：第一章/第一节</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>知识分类</t>
+          <t>题型</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -788,14 +704,14 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>用 / 分隔多级分类，例如：模块/章节/小节</t>
+          <t>只能填写：单选、多选、判断、简答</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>题型</t>
+          <t>题干</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -805,14 +721,14 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>只能填写：单选、多选、判断、简答</t>
+          <t>题目正文</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>选项A-D</t>
+          <t>A-D</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -822,14 +738,14 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>判断题和简答题可留空；选项E/F为兼容不定项题的可选扩展列</t>
+          <t>判断题可填写 正确/错误；简答题可留空</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>标准答案</t>
+          <t>正确答案</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -839,7 +755,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>单选填 A/B/C/D；多选填 ABC/ABD；判断填 对/错；简答填参考答案文本</t>
+          <t>单选填 A/B/C/D；多选填 ABC/ABD；判断填 正确/错误 或 对/错；简答填参考答案文本</t>
         </is>
       </c>
     </row>
@@ -857,6 +773,23 @@
       <c r="C7" t="inlineStr">
         <is>
           <t>题目解析或背诵要点</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>易错点标签</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>可用 、 或 , 分隔多个标签</t>
         </is>
       </c>
     </row>

</xml_diff>